<commit_message>
refactor(abilities)!: unify activation behavior through startup tasks
Resolve startup Instant effects and chained abilities synchronously in definition order, using an explicit stack for nested activation.

Replace activation_effects and end_on_activation with explicit effect and EndAbility tasks. Migrate configuration tables, generated code, call sites, tests, and documentation.

BREAKING CHANGE: GameplayAbility::new now takes five arguments, the removed fields and their APIs are unavailable, and configuration packages must be regenerated.
</commit_message>
<xml_diff>
--- a/config/tables/gas.ability.xlsx
+++ b/config/tables/gas.ability.xlsx
@@ -339,15 +339,13 @@
     <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="23" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="23" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -370,30 +368,24 @@
         <x:v>cooldown_effect_id</x:v>
       </x:c>
       <x:c r="G1" s="7" t="str">
-        <x:v>activation_effect_ids</x:v>
+        <x:v>asset_tags</x:v>
       </x:c>
       <x:c r="H1" s="7" t="str">
-        <x:v>asset_tags</x:v>
+        <x:v>required_tags</x:v>
       </x:c>
       <x:c r="I1" s="7" t="str">
-        <x:v>required_tags</x:v>
+        <x:v>blocked_tags</x:v>
       </x:c>
       <x:c r="J1" s="7" t="str">
-        <x:v>blocked_tags</x:v>
+        <x:v>cancel_ability_tags</x:v>
       </x:c>
       <x:c r="K1" s="7" t="str">
-        <x:v>cancel_ability_tags</x:v>
+        <x:v>block_ability_tags</x:v>
       </x:c>
       <x:c r="L1" s="7" t="str">
-        <x:v>block_ability_tags</x:v>
+        <x:v>targeting_id</x:v>
       </x:c>
       <x:c r="M1" s="7" t="str">
-        <x:v>targeting_id</x:v>
-      </x:c>
-      <x:c r="N1" s="7" t="str">
-        <x:v>end_on_activation</x:v>
-      </x:c>
-      <x:c r="O1" s="7" t="str">
         <x:v>allow_multiple_instances</x:v>
       </x:c>
     </x:row>
@@ -417,7 +409,7 @@
         <x:v>int?#ref=gas.TbEffect</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
-        <x:v>(list#sep=;),int#ref=gas.TbEffect</x:v>
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
         <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
@@ -432,15 +424,9 @@
         <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
       </x:c>
       <x:c r="L2" s="9" t="str">
-        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+        <x:v>int#ref=gas.TbTargeting</x:v>
       </x:c>
       <x:c r="M2" s="9" t="str">
-        <x:v>int#ref=gas.TbTargeting</x:v>
-      </x:c>
-      <x:c r="N2" s="9" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="O2" s="9" t="str">
         <x:v>bool</x:v>
       </x:c>
     </x:row>
@@ -460,8 +446,6 @@
       <x:c r="K3" s="8"/>
       <x:c r="L3" s="8"/>
       <x:c r="M3" s="8"/>
-      <x:c r="N3" s="8"/>
-      <x:c r="O3" s="8"/>
     </x:row>
     <x:row r="4" ht="66" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -483,30 +467,24 @@
         <x:v>Cooldown effect identifier. Blank means no cooldown.</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str">
-        <x:v>Effects applied to all captured activation targets, in listed order.</x:v>
+        <x:v>Ability identity tags separated by semicolons.</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
-        <x:v>Ability identity tags separated by semicolons.</x:v>
+        <x:v>Owner tags required for activation.</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
-        <x:v>Owner tags required for activation.</x:v>
+        <x:v>Owner tags that prevent activation.</x:v>
       </x:c>
       <x:c r="J4" s="11" t="str">
-        <x:v>Owner tags that prevent activation.</x:v>
+        <x:v>Active ability tags canceled on activation.</x:v>
       </x:c>
       <x:c r="K4" s="11" t="str">
-        <x:v>Active ability tags canceled on activation.</x:v>
+        <x:v>Ability tags blocked while this ability is active.</x:v>
       </x:c>
       <x:c r="L4" s="11" t="str">
-        <x:v>Ability tags blocked while this ability is active.</x:v>
+        <x:v>Targeting definition identifier.</x:v>
       </x:c>
       <x:c r="M4" s="11" t="str">
-        <x:v>Targeting definition identifier.</x:v>
-      </x:c>
-      <x:c r="N4" s="11" t="str">
-        <x:v>End the ability immediately after activation.</x:v>
-      </x:c>
-      <x:c r="O4" s="11" t="str">
         <x:v>Allow concurrent instances of this ability.</x:v>
       </x:c>
     </x:row>
@@ -527,32 +505,25 @@
       <x:c r="F5" s="12" t="n">
         <x:v>2002</x:v>
       </x:c>
-      <x:c r="G5" s="13"/>
-      <x:c r="H5" s="13" t="str">
+      <x:c r="G5" s="13" t="str">
         <x:v>Ability.Fireball</x:v>
       </x:c>
-      <x:c r="I5" s="13"/>
-      <x:c r="J5" s="13" t="str">
+      <x:c r="H5" s="13"/>
+      <x:c r="I5" s="13" t="str">
         <x:v>Cooldown.Fireball;State.Stunned</x:v>
       </x:c>
+      <x:c r="J5" s="13"/>
       <x:c r="K5" s="13"/>
-      <x:c r="L5" s="13"/>
-      <x:c r="M5" s="12" t="n">
+      <x:c r="L5" s="12" t="n">
         <x:v>3001</x:v>
       </x:c>
-      <x:c r="N5" s="5" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O5" s="5" t="b">
+      <x:c r="M5" s="5" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="N5">
-      <x:formula1>"TRUE,FALSE"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="O5">
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="M5">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
refactor(config)!: move child references into parent tables
Abilities reference ordered task and additional-cost IDs, while effects
reference ordered modifier IDs. Remove child owner and order fields,
and place additional_cost_ids immediately after cost_effect_id.

Update configuration compilation, validation, reports, documentation,
and regression coverage for ordering, sharing, and invalid references.

BREAKING CHANGE: The generated table schema and binary layout changed.
Re-export configuration data with the matching generated code.

Validation:
- config/export.ps1 and Luban validation
- cargo fmt
- cargo clippy --all-targets --all-features -- -D warnings
- cargo build
- cargo test --lib --tests -j 1 (210 passed, 1 ignored)
- cargo test --all-features --test config_test -j 1 (30 passed)
</commit_message>
<xml_diff>
--- a/config/tables/gas.ability.xlsx
+++ b/config/tables/gas.ability.xlsx
@@ -2,128 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ability" sheetId="1" r:id="Rbf343fdc7f3840fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ability" sheetId="1" r:id="Rdb0d7700c6064112"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">##var</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">id</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">name</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">max_level</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cost_effect_id</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cooldown_effect_id</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">asset_tags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">required_tags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">blocked_tags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cancel_ability_tags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">block_ability_tags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">targeting_id</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">allow_multiple_instances</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">##type</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">int#range=[1,1000000]</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">string</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">int#range=[1,100]</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">int?#ref=gas.TbEffect</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">(list#sep=;),string#ref=gas.TbTag</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">int#ref=gas.TbTargeting</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">bool</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">##group</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">##</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unique ability identifier.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Designer ability name.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Highest supported ability level.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cost effect identifier. Blank means no cost.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cooldown effect identifier. Blank means no cooldown.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ability identity tags separated by semicolons.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Owner tags required for activation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Owner tags that prevent activation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Active ability tags canceled on activation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ability tags blocked while this ability is active.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Targeting definition identifier.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Allow concurrent instances of this ability.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Fireball</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ability.Fireball</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cooldown.Fireball;State.Stunned</x:t>
-  </x:si>
-</x:sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1174,97 +1059,121 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" customWidth="1"/>
-    <x:col min="2" max="2" width="14" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="12" width="23" customWidth="1"/>
-    <x:col min="13" max="13" width="28" customWidth="1"/>
+    <x:col min="13" max="13" width="23" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="1" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D1" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F1" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G1" s="1" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="H1" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="I1" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="J1" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="K1" s="1" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L1" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="M1" s="1" t="s">
-        <x:v>12</x:v>
+      <x:c r="A1" s="1" t="str">
+        <x:v>##var</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="str">
+        <x:v>max_level</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="str">
+        <x:v>cost_effect_id</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="str">
+        <x:v>additional_cost_ids</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="str">
+        <x:v>cooldown_effect_id</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="str">
+        <x:v>asset_tags</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="str">
+        <x:v>required_tags</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="str">
+        <x:v>blocked_tags</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="str">
+        <x:v>cancel_ability_tags</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="str">
+        <x:v>block_ability_tags</x:v>
+      </x:c>
+      <x:c r="M1" s="1" t="str">
+        <x:v>targeting_id</x:v>
+      </x:c>
+      <x:c r="N1" s="1" t="str">
+        <x:v>allow_multiple_instances</x:v>
+      </x:c>
+      <x:c r="O1" s="1" t="str">
+        <x:v>task_ids</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="52" customHeight="1">
-      <x:c r="A2" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C2" s="2" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D2" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E2" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F2" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G2" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="H2" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I2" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="J2" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="K2" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="L2" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="M2" s="2" t="s">
-        <x:v>20</x:v>
+      <x:c r="A2" s="2" t="str">
+        <x:v>##type</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>int#range=[1,1000000]</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="str">
+        <x:v>int#range=[1,100]</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
+        <x:v>int?#ref=gas.TbEffect</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="str">
+        <x:v>(list#sep=;),(int#ref=gas.TbAbilityAdditionalCost)</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="str">
+        <x:v>int?#ref=gas.TbEffect</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="str">
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="str">
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="str">
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="str">
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="str">
+        <x:v>(list#sep=;),string#ref=gas.TbTag</x:v>
+      </x:c>
+      <x:c r="M2" s="2" t="str">
+        <x:v>int#ref=gas.TbTargeting</x:v>
+      </x:c>
+      <x:c r="N2" s="2" t="str">
+        <x:v>bool</x:v>
+      </x:c>
+      <x:c r="O2" s="2" t="str">
+        <x:v>(list#sep=;),(int#ref=gas.TbAbilityTask)</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="A3" s="3" t="str">
+        <x:v>##group</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -1278,79 +1187,91 @@
       <x:c r="K3" s="3"/>
       <x:c r="L3" s="3"/>
       <x:c r="M3" s="3"/>
+      <x:c r="N3" s="3"/>
+      <x:c r="O3" s="3"/>
     </x:row>
     <x:row r="4" ht="66" customHeight="1">
-      <x:c r="A4" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D4" s="4" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F4" s="4" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="G4" s="4" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="H4" s="4" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="I4" s="4" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J4" s="4" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="K4" s="4" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="L4" s="4" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="M4" s="4" t="s">
-        <x:v>34</x:v>
+      <x:c r="A4" s="4" t="str">
+        <x:v>##</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="str">
+        <x:v>Unique ability identifier.</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="str">
+        <x:v>Designer ability name.</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="str">
+        <x:v>Highest supported ability level.</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="str">
+        <x:v>Cost effect identifier. Blank means no cost.</x:v>
+      </x:c>
+      <x:c r="F4" s="4" t="str">
+        <x:v>Additional cost IDs in payment order. Blank means none.</x:v>
+      </x:c>
+      <x:c r="G4" s="4" t="str">
+        <x:v>Cooldown effect identifier. Blank means no cooldown.</x:v>
+      </x:c>
+      <x:c r="H4" s="4" t="str">
+        <x:v>Ability identity tags separated by semicolons.</x:v>
+      </x:c>
+      <x:c r="I4" s="4" t="str">
+        <x:v>Owner tags required for activation.</x:v>
+      </x:c>
+      <x:c r="J4" s="4" t="str">
+        <x:v>Owner tags that prevent activation.</x:v>
+      </x:c>
+      <x:c r="K4" s="4" t="str">
+        <x:v>Active ability tags canceled on activation.</x:v>
+      </x:c>
+      <x:c r="L4" s="4" t="str">
+        <x:v>Ability tags blocked while this ability is active.</x:v>
+      </x:c>
+      <x:c r="M4" s="4" t="str">
+        <x:v>Targeting definition identifier.</x:v>
+      </x:c>
+      <x:c r="N4" s="4" t="str">
+        <x:v>Allow concurrent instances of this ability.</x:v>
+      </x:c>
+      <x:c r="O4" s="4" t="str">
+        <x:v>Task IDs. Same-tick actions follow list order.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
       <x:c r="A5" s="5"/>
-      <x:c r="B5" s="6">
+      <x:c r="B5" s="6" t="n">
         <x:v>1001</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="D5" s="6">
+      <x:c r="C5" s="7" t="str">
+        <x:v>Fireball</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="6">
+      <x:c r="E5" s="6" t="n">
         <x:v>2001</x:v>
       </x:c>
-      <x:c r="F5" s="6">
+      <x:c r="F5" s="7"/>
+      <x:c r="G5" s="6" t="n">
         <x:v>2002</x:v>
       </x:c>
-      <x:c r="G5" s="7" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="J5" s="7"/>
+      <x:c r="H5" s="7" t="str">
+        <x:v>Ability.Fireball</x:v>
+      </x:c>
+      <x:c r="I5" s="7"/>
+      <x:c r="J5" s="7" t="str">
+        <x:v>Cooldown.Fireball;State.Stunned</x:v>
+      </x:c>
       <x:c r="K5" s="7"/>
-      <x:c r="L5" s="6">
+      <x:c r="L5" s="7"/>
+      <x:c r="M5" s="6" t="n">
         <x:v>3001</x:v>
       </x:c>
-      <x:c r="M5" s="5" t="b">
+      <x:c r="N5" s="5" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="O5" s="7" t="str">
+        <x:v>10011;10012</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -1367,25 +1288,31 @@
       <x:c r="E6" s="13" t="n">
         <x:v>2001</x:v>
       </x:c>
-      <x:c r="F6" s="13"/>
-      <x:c r="G6" s="14"/>
+      <x:c r="F6" s="14" t="str">
+        <x:v>10021</x:v>
+      </x:c>
+      <x:c r="G6" s="13"/>
       <x:c r="H6" s="14"/>
       <x:c r="I6" s="14"/>
       <x:c r="J6" s="14"/>
       <x:c r="K6" s="14"/>
-      <x:c r="L6" s="13" t="n">
+      <x:c r="L6" s="14"/>
+      <x:c r="M6" s="13" t="n">
         <x:v>3001</x:v>
       </x:c>
-      <x:c r="M6" s="12" t="b">
+      <x:c r="N6" s="12" t="b">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="O6" s="14" t="str">
+        <x:v>10021</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="M5">
+    <x:dataValidation type="list" sqref="N5">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M6">
+    <x:dataValidation type="list" sqref="N6">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>